<commit_message>
feat: agrega prospectos gomas/motos Floresta-Devoto - 2026-06-26
</commit_message>
<xml_diff>
--- a/Prospectos_CABA.xlsx
+++ b/Prospectos_CABA.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M212"/>
+  <dimension ref="A1:M216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10197,6 +10197,186 @@
       </c>
       <c r="M212" s="3" t="inlineStr"/>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Gomería José</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Gomería / Neumáticos para motos</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Av. Rivadavia 8911, Floresta, CABA</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>+54 11 2353-8799</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/neumaticos_jg</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>ciclolandiamotos.com.ar</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Sin sitio web propio. Solo Instagram @neumaticos_jg</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Moto Service Devoto</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Taller mecánico de motos</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Av. San Martín 7411, Villa Devoto, CABA</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/motoservicedevoto</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>ciclolandiamotos.com.ar / fulltimemotos.com.ar</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Sin sitio web propio. Solo Instagram @motoservicedevoto. Calificación 10/10 con 68 reseñas. Responsable: Sebastián</t>
+        </is>
+      </c>
+      <c r="K214" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Taller Osvaldo Mecánica General</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Taller mecánico de motos</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Euclides 4878, Floresta, CABA</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>011 1168-1475</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>argentino.com.ar</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Sin sitio web propio. Solo aparece en directorios. Ofrece inyección electrónica y diagnóstico</t>
+        </is>
+      </c>
+      <c r="K215" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>FC Taller de Motos</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Taller mecánico de motos</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>CABA (zona Floresta)</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Taller-mecanico-de-motos-FC-108898608458725</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fctallerdemotos</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Instagram / Facebook</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Sin sitio web propio. Solo redes sociales. Dirección exacta pendiente de confirmar</t>
+        </is>
+      </c>
+      <c r="K216" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: reinserta prospectos motos Floresta-Devoto con formato correcto
</commit_message>
<xml_diff>
--- a/Prospectos_CABA.xlsx
+++ b/Prospectos_CABA.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +32,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +56,13 @@
         <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -75,11 +84,25 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,6 +119,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10198,183 +10223,195 @@
       <c r="M212" s="3" t="inlineStr"/>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr">
+      <c r="A213" s="6" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" s="6" t="inlineStr">
         <is>
           <t>Gomería José</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="C213" s="6" t="inlineStr">
         <is>
           <t>Gomería / Neumáticos para motos</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>Floresta</t>
+        </is>
+      </c>
+      <c r="E213" s="6" t="inlineStr">
         <is>
           <t>Av. Rivadavia 8911, Floresta, CABA</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
+      <c r="F213" s="6" t="inlineStr">
         <is>
           <t>+54 11 2353-8799</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/neumaticos_jg</t>
-        </is>
-      </c>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>ciclolandiamotos.com.ar</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>Sin sitio web propio. Solo Instagram @neumaticos_jg</t>
-        </is>
-      </c>
-      <c r="K213" t="n">
-        <v>3</v>
+      <c r="G213" s="6" t="inlineStr">
+        <is>
+          <t>+54 11 2353-8799</t>
+        </is>
+      </c>
+      <c r="H213" s="6" t="n"/>
+      <c r="I213" s="6" t="inlineStr">
+        <is>
+          <t>@neumaticos_jg</t>
+        </is>
+      </c>
+      <c r="J213" s="6" t="n"/>
+      <c r="K213" s="6" t="n"/>
+      <c r="L213" s="6" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="M213" s="6" t="inlineStr">
+        <is>
+          <t>Sin sitio web propio. Solo Instagram</t>
+        </is>
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="inlineStr">
+      <c r="A214" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" s="7" t="inlineStr">
         <is>
           <t>Moto Service Devoto</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
+      <c r="C214" s="7" t="inlineStr">
         <is>
           <t>Taller mecánico de motos</t>
         </is>
       </c>
-      <c r="C214" t="inlineStr">
+      <c r="D214" s="7" t="inlineStr">
+        <is>
+          <t>Villa Devoto</t>
+        </is>
+      </c>
+      <c r="E214" s="7" t="inlineStr">
         <is>
           <t>Av. San Martín 7411, Villa Devoto, CABA</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/motoservicedevoto</t>
-        </is>
-      </c>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>ciclolandiamotos.com.ar / fulltimemotos.com.ar</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>Sin sitio web propio. Solo Instagram @motoservicedevoto. Calificación 10/10 con 68 reseñas. Responsable: Sebastián</t>
-        </is>
-      </c>
-      <c r="K214" t="n">
-        <v>3</v>
+      <c r="F214" s="7" t="n"/>
+      <c r="G214" s="7" t="n"/>
+      <c r="H214" s="7" t="n"/>
+      <c r="I214" s="7" t="inlineStr">
+        <is>
+          <t>@motoservicedevoto</t>
+        </is>
+      </c>
+      <c r="J214" s="7" t="n"/>
+      <c r="K214" s="7" t="n"/>
+      <c r="L214" s="7" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="M214" s="7" t="inlineStr">
+        <is>
+          <t>Sin sitio web. Solo Instagram. Calificación 10/10 (68 reseñas). Responsable: Sebastián</t>
+        </is>
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr">
+      <c r="A215" s="6" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" s="6" t="inlineStr">
         <is>
           <t>Taller Osvaldo Mecánica General</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
+      <c r="C215" s="6" t="inlineStr">
         <is>
           <t>Taller mecánico de motos</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t>Floresta</t>
+        </is>
+      </c>
+      <c r="E215" s="6" t="inlineStr">
         <is>
           <t>Euclides 4878, Floresta, CABA</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr">
+      <c r="F215" s="6" t="inlineStr">
         <is>
           <t>011 1168-1475</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr">
-        <is>
-          <t>argentino.com.ar</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>Sin sitio web propio. Solo aparece en directorios. Ofrece inyección electrónica y diagnóstico</t>
-        </is>
-      </c>
-      <c r="K215" t="n">
-        <v>3</v>
+      <c r="G215" s="6" t="n"/>
+      <c r="H215" s="6" t="n"/>
+      <c r="I215" s="6" t="n"/>
+      <c r="J215" s="6" t="n"/>
+      <c r="K215" s="6" t="n"/>
+      <c r="L215" s="6" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="M215" s="6" t="inlineStr">
+        <is>
+          <t>Sin web. Solo aparece en directorios. Inyección electrónica y diagnóstico</t>
+        </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr">
+      <c r="A216" s="7" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" s="7" t="inlineStr">
         <is>
           <t>FC Taller de Motos</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
+      <c r="C216" s="7" t="inlineStr">
         <is>
           <t>Taller mecánico de motos</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>CABA (zona Floresta)</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/Taller-mecanico-de-motos-FC-108898608458725</t>
-        </is>
-      </c>
-      <c r="G216" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fctallerdemotos</t>
-        </is>
-      </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>Instagram / Facebook</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>Sin sitio web propio. Solo redes sociales. Dirección exacta pendiente de confirmar</t>
-        </is>
-      </c>
-      <c r="K216" t="n">
-        <v>3</v>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t>Floresta</t>
+        </is>
+      </c>
+      <c r="E216" s="7" t="inlineStr">
+        <is>
+          <t>CABA (zona Floresta - confirmar dirección)</t>
+        </is>
+      </c>
+      <c r="F216" s="7" t="n"/>
+      <c r="G216" s="7" t="n"/>
+      <c r="H216" s="7" t="inlineStr">
+        <is>
+          <t>@fctallerdemotos</t>
+        </is>
+      </c>
+      <c r="I216" s="7" t="inlineStr">
+        <is>
+          <t>@fctallerdemotos</t>
+        </is>
+      </c>
+      <c r="J216" s="7" t="n"/>
+      <c r="K216" s="7" t="n"/>
+      <c r="L216" s="7" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="M216" s="7" t="inlineStr">
+        <is>
+          <t>Sin web. Solo Facebook e Instagram. Dirección exacta pendiente de confirmar</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>